<commit_message>
working discount modwls with random demand variation
</commit_message>
<xml_diff>
--- a/Deterministic/Model Files/Segment Test/data/Starting_point.xlsx
+++ b/Deterministic/Model Files/Segment Test/data/Starting_point.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uark-my.sharepoint.com/personal/uhorchak_uark_edu/Documents/Desktop/Vaccine_Tender/Model Files/L-Shaped/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uark-my.sharepoint.com/personal/uhorchak_uark_edu/Documents/Desktop/Vaccine_Tender/Deterministic/Model Files/Segment Test/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3531FE4D-4523-48B9-AC88-B1CF65308B73}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{FA3337A2-F403-407B-92A1-0BBD98A29972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98964434-48BB-4FCC-96EC-352152809D98}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -253,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -262,9 +262,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -272,8 +269,14 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -290,6 +293,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -673,7 +680,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" t="s">
         <v>2</v>
       </c>
       <c r="B11">
@@ -718,7 +725,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E851515-DB43-462D-9C92-F50748C0A12A}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -727,7 +734,7 @@
     <col min="5" max="5" width="16.109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -744,7 +751,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -757,11 +764,12 @@
       <c r="D2" s="2">
         <v>3</v>
       </c>
-      <c r="E2" s="4">
-        <v>13299</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E2" s="7">
+        <v>132990009</v>
+      </c>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -774,11 +782,12 @@
       <c r="D3" s="2">
         <v>3</v>
       </c>
-      <c r="E3" s="3">
-        <v>12505</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E3" s="8">
+        <v>785050009</v>
+      </c>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -791,11 +800,13 @@
       <c r="D4" s="2">
         <v>3</v>
       </c>
-      <c r="E4" s="3">
-        <v>13547</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E4" s="8">
+        <v>98611200099</v>
+      </c>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -808,11 +819,12 @@
       <c r="D5" s="2">
         <v>3</v>
       </c>
-      <c r="E5" s="4">
-        <v>6547</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E5" s="7">
+        <v>9959800009</v>
+      </c>
+      <c r="F5" s="9"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -825,11 +837,12 @@
       <c r="D6" s="2">
         <v>3</v>
       </c>
-      <c r="E6" s="4">
-        <v>90279</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E6" s="7">
+        <v>902790009</v>
+      </c>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -842,11 +855,12 @@
       <c r="D7" s="2">
         <v>1</v>
       </c>
-      <c r="E7" s="4">
-        <v>180177</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E7" s="7">
+        <v>180177000</v>
+      </c>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -859,11 +873,12 @@
       <c r="D8" s="2">
         <v>1</v>
       </c>
-      <c r="E8" s="4">
-        <v>13305</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E8" s="7">
+        <v>13305000</v>
+      </c>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
@@ -876,11 +891,12 @@
       <c r="D9" s="2">
         <v>1</v>
       </c>
-      <c r="E9" s="4">
-        <v>8948</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E9" s="7">
+        <v>8948000</v>
+      </c>
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -893,11 +909,12 @@
       <c r="D10" s="2">
         <v>1</v>
       </c>
-      <c r="E10" s="4">
-        <v>140932</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E10" s="7">
+        <v>140932000</v>
+      </c>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -910,11 +927,12 @@
       <c r="D11" s="2">
         <v>1</v>
       </c>
-      <c r="E11" s="4">
-        <v>17896</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E11" s="7">
+        <v>17896000</v>
+      </c>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -927,11 +945,12 @@
       <c r="D12" s="2">
         <v>1</v>
       </c>
-      <c r="E12" s="4">
-        <v>31318</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E12" s="7">
+        <v>31318000</v>
+      </c>
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -944,11 +963,12 @@
       <c r="D13" s="2">
         <v>1</v>
       </c>
-      <c r="E13" s="4">
-        <v>53688</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E13" s="7">
+        <v>53688000</v>
+      </c>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -961,11 +981,12 @@
       <c r="D14" s="2">
         <v>1</v>
       </c>
-      <c r="E14" s="4">
-        <v>43365</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E14" s="7">
+        <v>43365000</v>
+      </c>
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -978,11 +999,12 @@
       <c r="D15" s="2">
         <v>1</v>
       </c>
-      <c r="E15" s="4">
-        <v>40214</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E15" s="7">
+        <v>40214000</v>
+      </c>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -995,11 +1017,12 @@
       <c r="D16" s="2">
         <v>1</v>
       </c>
-      <c r="E16" s="4">
-        <v>219201</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E16" s="7">
+        <v>219201000</v>
+      </c>
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -1012,11 +1035,12 @@
       <c r="D17" s="2">
         <v>1</v>
       </c>
-      <c r="E17" s="4">
-        <v>61221</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E17" s="7">
+        <v>61221000</v>
+      </c>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
@@ -1029,11 +1053,12 @@
       <c r="D18" s="2">
         <v>1</v>
       </c>
-      <c r="E18" s="4">
-        <v>84681</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E18" s="7">
+        <v>84681000</v>
+      </c>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -1046,11 +1071,12 @@
       <c r="D19" s="2">
         <v>5</v>
       </c>
-      <c r="E19" s="4">
-        <v>3625</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E19" s="7">
+        <v>3625000</v>
+      </c>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1063,11 +1089,12 @@
       <c r="D20" s="2">
         <v>5</v>
       </c>
-      <c r="E20" s="4">
-        <v>13464</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E20" s="7">
+        <v>13464000</v>
+      </c>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
@@ -1080,11 +1107,12 @@
       <c r="D21" s="2">
         <v>5</v>
       </c>
-      <c r="E21" s="4">
-        <v>5391</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E21" s="7">
+        <v>5391000</v>
+      </c>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
@@ -1097,11 +1125,12 @@
       <c r="D22" s="2">
         <v>1</v>
       </c>
-      <c r="E22" s="4">
-        <v>56510</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E22" s="7">
+        <v>56510000</v>
+      </c>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>10</v>
       </c>
@@ -1114,11 +1143,12 @@
       <c r="D23" s="2">
         <v>1</v>
       </c>
-      <c r="E23" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E23" s="7">
+        <v>63514000</v>
+      </c>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -1131,11 +1161,12 @@
       <c r="D24" s="2">
         <v>1</v>
       </c>
-      <c r="E24" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E24" s="7">
+        <v>25642000</v>
+      </c>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>13</v>
       </c>
@@ -1148,11 +1179,12 @@
       <c r="D25" s="2">
         <v>3</v>
       </c>
-      <c r="E25" s="4">
-        <v>185663</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E25" s="7">
+        <v>25642000</v>
+      </c>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>13</v>
       </c>
@@ -1165,11 +1197,12 @@
       <c r="D26" s="2">
         <v>3</v>
       </c>
-      <c r="E26" s="4">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E26" s="7">
+        <v>25642000</v>
+      </c>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
@@ -1182,26 +1215,29 @@
       <c r="D27" s="2">
         <v>3</v>
       </c>
-      <c r="E27" s="4">
-        <v>148533</v>
-      </c>
+      <c r="E27" s="7">
+        <v>25642000</v>
+      </c>
+      <c r="F27" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF8CA8F-1DBE-42B3-8633-48C2ED5062E9}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1209,139 +1245,140 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <v>398056107.80000001</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>27968660.210000001</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>410128001.42000002</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="8">
-        <v>590379508</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="10">
+        <v>9876337950899990</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="8">
-        <v>280763726</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="10">
+        <v>9987637269</v>
+      </c>
+      <c r="C6" s="9"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="8">
-        <v>879375105</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B7" s="10">
+        <v>11576375105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="8">
-        <v>83171840</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="10">
+        <v>139131718409</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="10">
         <v>7682600</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="10">
         <v>3278988.3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="10">
         <v>2828944.58</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="10">
         <v>116834378.34999999</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="10">
         <v>5298997.59</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="10">
         <v>30290394.390000001</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="10">
         <v>43271991.979999997</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="10">
         <v>86543983.959999993</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="8">
-        <v>242285505</v>
+      <c r="B17" s="10">
+        <v>442285505</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="10">
         <v>156726900</v>
       </c>
     </row>
@@ -1364,7 +1401,7 @@
       <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1372,7 +1409,7 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1380,7 +1417,7 @@
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1388,7 +1425,7 @@
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1396,7 +1433,7 @@
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1404,7 +1441,7 @@
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1412,7 +1449,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1420,7 +1457,7 @@
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1428,7 +1465,7 @@
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1436,7 +1473,7 @@
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1444,7 +1481,7 @@
       <c r="A11" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1452,7 +1489,7 @@
       <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1460,7 +1497,7 @@
       <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>